<commit_message>
Mise à jour site Bois
</commit_message>
<xml_diff>
--- a/prix/prix.xlsx
+++ b/prix/prix.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\bois\prix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6CD674D-8219-4D60-911E-DB2EF4C92697}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A98CCFC-8FD7-4846-8953-66AB40EBEF48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="19416" windowHeight="11016" xr2:uid="{6E95DC93-531D-460D-9A06-44397A8920D7}"/>
   </bookViews>
@@ -1514,7 +1514,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
@@ -1584,43 +1584,6 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -2000,13 +1963,13 @@
       <c r="C2" s="2" t="s">
         <v>341</v>
       </c>
-      <c r="D2" s="25">
+      <c r="D2" s="11">
         <v>15.44</v>
       </c>
       <c r="E2" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="26">
+      <c r="F2" s="12">
         <v>117.38500000000023</v>
       </c>
     </row>
@@ -2020,13 +1983,13 @@
       <c r="C3" s="2" t="s">
         <v>342</v>
       </c>
-      <c r="D3" s="25">
+      <c r="D3" s="11">
         <v>18.73</v>
       </c>
       <c r="E3" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="F3" s="26">
+      <c r="F3" s="12">
         <v>0</v>
       </c>
     </row>
@@ -2040,13 +2003,13 @@
       <c r="C4" s="2" t="s">
         <v>313</v>
       </c>
-      <c r="D4" s="25">
+      <c r="D4" s="11">
         <v>8.81</v>
       </c>
       <c r="E4" s="19" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="26">
+      <c r="F4" s="12">
         <v>343.69899999999916</v>
       </c>
     </row>
@@ -2060,13 +2023,13 @@
       <c r="C5" s="2" t="s">
         <v>314</v>
       </c>
-      <c r="D5" s="25">
+      <c r="D5" s="11">
         <v>10.78</v>
       </c>
       <c r="E5" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="26">
+      <c r="F5" s="12">
         <v>385.91999999999973</v>
       </c>
     </row>
@@ -2080,13 +2043,13 @@
       <c r="C6" s="2" t="s">
         <v>316</v>
       </c>
-      <c r="D6" s="25">
+      <c r="D6" s="11">
         <v>12.41</v>
       </c>
       <c r="E6" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="26">
+      <c r="F6" s="12">
         <v>443.51999999999975</v>
       </c>
     </row>
@@ -2100,13 +2063,13 @@
       <c r="C7" s="2" t="s">
         <v>315</v>
       </c>
-      <c r="D7" s="25">
+      <c r="D7" s="11">
         <v>15.74</v>
       </c>
       <c r="E7" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="F7" s="26">
+      <c r="F7" s="12">
         <v>119.51800000000065</v>
       </c>
     </row>
@@ -2115,13 +2078,13 @@
       <c r="B8" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="D8" s="25">
+      <c r="D8" s="11">
         <v>14.71</v>
       </c>
       <c r="E8" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="26">
+      <c r="F8" s="12">
         <v>45</v>
       </c>
     </row>
@@ -2130,13 +2093,13 @@
       <c r="B9" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="D9" s="25">
+      <c r="D9" s="11">
         <v>21.56</v>
       </c>
       <c r="E9" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="26">
+      <c r="F9" s="12">
         <v>-3.5527136788005009E-15</v>
       </c>
     </row>
@@ -2145,13 +2108,13 @@
       <c r="B10" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="D10" s="25">
+      <c r="D10" s="11">
         <v>44.06</v>
       </c>
       <c r="E10" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="F10" s="26">
+      <c r="F10" s="12">
         <v>11.519999999999982</v>
       </c>
     </row>
@@ -2160,13 +2123,13 @@
       <c r="B11" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="D11" s="25">
+      <c r="D11" s="11">
         <v>91.48</v>
       </c>
       <c r="E11" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="F11" s="26">
+      <c r="F11" s="12">
         <v>0</v>
       </c>
     </row>
@@ -2175,13 +2138,13 @@
       <c r="B12" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="D12" s="25">
+      <c r="D12" s="11">
         <v>2.31</v>
       </c>
       <c r="E12" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="F12" s="26">
+      <c r="F12" s="12">
         <v>0</v>
       </c>
     </row>
@@ -2195,13 +2158,13 @@
       <c r="C13" s="2" t="s">
         <v>317</v>
       </c>
-      <c r="D13" s="25">
+      <c r="D13" s="11">
         <v>7.79</v>
       </c>
       <c r="E13" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="F13" s="26">
+      <c r="F13" s="12">
         <v>14.900000000000224</v>
       </c>
     </row>
@@ -2215,13 +2178,13 @@
       <c r="C14" s="2" t="s">
         <v>318</v>
       </c>
-      <c r="D14" s="25">
+      <c r="D14" s="11">
         <v>10.83</v>
       </c>
       <c r="E14" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="F14" s="26">
+      <c r="F14" s="12">
         <v>32.024999999999835</v>
       </c>
     </row>
@@ -2235,13 +2198,13 @@
       <c r="C15" s="2" t="s">
         <v>319</v>
       </c>
-      <c r="D15" s="25">
+      <c r="D15" s="11">
         <v>13.94</v>
       </c>
       <c r="E15" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="F15" s="26">
+      <c r="F15" s="12">
         <v>12.150000000000212</v>
       </c>
     </row>
@@ -2255,13 +2218,13 @@
       <c r="C16" s="2" t="s">
         <v>320</v>
       </c>
-      <c r="D16" s="25">
+      <c r="D16" s="11">
         <v>0</v>
       </c>
       <c r="E16" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="F16" s="26">
+      <c r="F16" s="12">
         <v>0</v>
       </c>
     </row>
@@ -2275,13 +2238,13 @@
       <c r="C17" s="2" t="s">
         <v>321</v>
       </c>
-      <c r="D17" s="25">
+      <c r="D17" s="11">
         <v>20.09</v>
       </c>
       <c r="E17" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="F17" s="26">
+      <c r="F17" s="12">
         <v>4.9999999981578114E-3</v>
       </c>
     </row>
@@ -2295,13 +2258,13 @@
       <c r="C18" s="2" t="s">
         <v>322</v>
       </c>
-      <c r="D18" s="25">
+      <c r="D18" s="11">
         <v>16.75</v>
       </c>
       <c r="E18" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="F18" s="26">
+      <c r="F18" s="12">
         <v>0</v>
       </c>
     </row>
@@ -2315,13 +2278,13 @@
       <c r="C19" s="2" t="s">
         <v>323</v>
       </c>
-      <c r="D19" s="25">
+      <c r="D19" s="11">
         <v>19.990000000000002</v>
       </c>
       <c r="E19" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="F19" s="26">
+      <c r="F19" s="12">
         <v>140.29799999999338</v>
       </c>
     </row>
@@ -2335,13 +2298,13 @@
       <c r="C20" s="5" t="s">
         <v>324</v>
       </c>
-      <c r="D20" s="25">
+      <c r="D20" s="11">
         <v>28.560000000000002</v>
       </c>
       <c r="E20" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="F20" s="26">
+      <c r="F20" s="12">
         <v>167.15000000000467</v>
       </c>
     </row>
@@ -2355,13 +2318,13 @@
       <c r="C21" s="5" t="s">
         <v>325</v>
       </c>
-      <c r="D21" s="25">
+      <c r="D21" s="11">
         <v>28.34</v>
       </c>
       <c r="E21" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="F21" s="26">
+      <c r="F21" s="12">
         <v>150.97200000000186</v>
       </c>
     </row>
@@ -2375,13 +2338,13 @@
       <c r="C22" s="2" t="s">
         <v>326</v>
       </c>
-      <c r="D22" s="25">
+      <c r="D22" s="11">
         <v>54.51</v>
       </c>
       <c r="E22" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="F22" s="26">
+      <c r="F22" s="12">
         <v>-4.9999999999914557E-3</v>
       </c>
     </row>
@@ -2395,13 +2358,13 @@
       <c r="C23" s="2" t="s">
         <v>327</v>
       </c>
-      <c r="D23" s="25">
+      <c r="D23" s="11">
         <v>39.340000000000003</v>
       </c>
       <c r="E23" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="F23" s="26">
+      <c r="F23" s="12">
         <v>0</v>
       </c>
     </row>
@@ -2415,13 +2378,13 @@
       <c r="C24" s="2" t="s">
         <v>328</v>
       </c>
-      <c r="D24" s="25">
+      <c r="D24" s="11">
         <v>9.4500000000000011</v>
       </c>
       <c r="E24" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="F24" s="26">
+      <c r="F24" s="12">
         <v>35.736999999999895</v>
       </c>
     </row>
@@ -2435,13 +2398,13 @@
       <c r="C25" s="2" t="s">
         <v>329</v>
       </c>
-      <c r="D25" s="25">
+      <c r="D25" s="11">
         <v>10.39</v>
       </c>
       <c r="E25" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="F25" s="26">
+      <c r="F25" s="12">
         <v>0</v>
       </c>
     </row>
@@ -2455,13 +2418,13 @@
       <c r="C26" s="2" t="s">
         <v>330</v>
       </c>
-      <c r="D26" s="25">
+      <c r="D26" s="11">
         <v>8.98</v>
       </c>
       <c r="E26" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="F26" s="26">
+      <c r="F26" s="12">
         <v>74.247999999999593</v>
       </c>
     </row>
@@ -2475,13 +2438,13 @@
       <c r="C27" s="2" t="s">
         <v>331</v>
       </c>
-      <c r="D27" s="25">
+      <c r="D27" s="11">
         <v>10.81</v>
       </c>
       <c r="E27" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="F27" s="26">
+      <c r="F27" s="12">
         <v>145.5270000000001</v>
       </c>
     </row>
@@ -2495,13 +2458,13 @@
       <c r="C28" s="2" t="s">
         <v>332</v>
       </c>
-      <c r="D28" s="25">
+      <c r="D28" s="11">
         <v>8.8000000000000007</v>
       </c>
       <c r="E28" s="19" t="s">
         <v>32</v>
       </c>
-      <c r="F28" s="26">
+      <c r="F28" s="12">
         <v>0</v>
       </c>
     </row>
@@ -2515,13 +2478,13 @@
       <c r="C29" s="2" t="s">
         <v>334</v>
       </c>
-      <c r="D29" s="25">
+      <c r="D29" s="11">
         <v>16.080000000000002</v>
       </c>
       <c r="E29" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="F29" s="26">
+      <c r="F29" s="12">
         <v>178.6339999999939</v>
       </c>
     </row>
@@ -2535,13 +2498,13 @@
       <c r="C30" s="2" t="s">
         <v>333</v>
       </c>
-      <c r="D30" s="25">
+      <c r="D30" s="11">
         <v>15.71</v>
       </c>
       <c r="E30" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="F30" s="26">
+      <c r="F30" s="12">
         <v>0</v>
       </c>
     </row>
@@ -2555,13 +2518,13 @@
       <c r="C31" s="2" t="s">
         <v>335</v>
       </c>
-      <c r="D31" s="25">
+      <c r="D31" s="11">
         <v>31.3</v>
       </c>
       <c r="E31" s="19" t="s">
         <v>35</v>
       </c>
-      <c r="F31" s="26">
+      <c r="F31" s="12">
         <v>0</v>
       </c>
     </row>
@@ -2575,13 +2538,13 @@
       <c r="C32" s="2" t="s">
         <v>336</v>
       </c>
-      <c r="D32" s="25">
+      <c r="D32" s="11">
         <v>31.3</v>
       </c>
       <c r="E32" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="F32" s="26">
+      <c r="F32" s="12">
         <v>0</v>
       </c>
     </row>
@@ -2595,13 +2558,13 @@
       <c r="C33" s="2" t="s">
         <v>340</v>
       </c>
-      <c r="D33" s="25">
+      <c r="D33" s="11">
         <v>12.98</v>
       </c>
       <c r="E33" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="F33" s="26">
+      <c r="F33" s="12">
         <v>152.56700000000018</v>
       </c>
     </row>
@@ -2615,13 +2578,13 @@
       <c r="C34" s="2" t="s">
         <v>339</v>
       </c>
-      <c r="D34" s="25">
+      <c r="D34" s="11">
         <v>18.11</v>
       </c>
       <c r="E34" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="F34" s="26">
+      <c r="F34" s="12">
         <v>169.2409999999937</v>
       </c>
     </row>
@@ -2635,13 +2598,13 @@
       <c r="C35" s="2" t="s">
         <v>337</v>
       </c>
-      <c r="D35" s="25">
+      <c r="D35" s="11">
         <v>18.97</v>
       </c>
       <c r="E35" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="F35" s="26">
+      <c r="F35" s="12">
         <v>0</v>
       </c>
     </row>
@@ -2655,13 +2618,13 @@
       <c r="C36" s="2" t="s">
         <v>343</v>
       </c>
-      <c r="D36" s="25">
+      <c r="D36" s="11">
         <v>24.560000000000002</v>
       </c>
       <c r="E36" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="F36" s="26">
+      <c r="F36" s="12">
         <v>0</v>
       </c>
     </row>
@@ -2675,13 +2638,13 @@
       <c r="C37" s="2" t="s">
         <v>344</v>
       </c>
-      <c r="D37" s="25">
+      <c r="D37" s="11">
         <v>56.24</v>
       </c>
       <c r="E37" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="F37" s="26">
+      <c r="F37" s="12">
         <v>0</v>
       </c>
     </row>
@@ -2695,13 +2658,13 @@
       <c r="C38" s="2" t="s">
         <v>345</v>
       </c>
-      <c r="D38" s="25">
+      <c r="D38" s="11">
         <v>91.48</v>
       </c>
       <c r="E38" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="F38" s="26">
+      <c r="F38" s="12">
         <v>0</v>
       </c>
     </row>
@@ -2715,13 +2678,13 @@
       <c r="C39" s="2" t="s">
         <v>338</v>
       </c>
-      <c r="D39" s="25">
+      <c r="D39" s="11">
         <v>30.060000000000002</v>
       </c>
       <c r="E39" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="F39" s="26">
+      <c r="F39" s="12">
         <v>87.61900000000422</v>
       </c>
     </row>
@@ -2730,13 +2693,13 @@
       <c r="B40" s="14" t="s">
         <v>112</v>
       </c>
-      <c r="D40" s="25">
+      <c r="D40" s="11">
         <v>34.82</v>
       </c>
       <c r="E40" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="F40" s="26">
+      <c r="F40" s="12">
         <v>0</v>
       </c>
     </row>
@@ -2745,13 +2708,13 @@
       <c r="B41" s="14" t="s">
         <v>113</v>
       </c>
-      <c r="D41" s="25">
+      <c r="D41" s="11">
         <v>16.64</v>
       </c>
       <c r="E41" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="F41" s="26">
+      <c r="F41" s="12">
         <v>0</v>
       </c>
     </row>
@@ -2760,13 +2723,13 @@
       <c r="B42" s="14" t="s">
         <v>114</v>
       </c>
-      <c r="D42" s="25">
+      <c r="D42" s="11">
         <v>24.72</v>
       </c>
       <c r="E42" s="19" t="s">
         <v>46</v>
       </c>
-      <c r="F42" s="26">
+      <c r="F42" s="12">
         <v>2.34</v>
       </c>
     </row>
@@ -2775,13 +2738,13 @@
       <c r="B43" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="D43" s="25">
+      <c r="D43" s="11">
         <v>25.16</v>
       </c>
       <c r="E43" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="F43" s="26">
+      <c r="F43" s="12">
         <v>4.3964831775156199E-14</v>
       </c>
     </row>
@@ -2790,13 +2753,13 @@
       <c r="B44" s="14" t="s">
         <v>116</v>
       </c>
-      <c r="D44" s="25">
+      <c r="D44" s="11">
         <v>28.8</v>
       </c>
       <c r="E44" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="F44" s="26">
+      <c r="F44" s="12">
         <v>0</v>
       </c>
     </row>
@@ -2805,13 +2768,13 @@
       <c r="B45" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="D45" s="25">
+      <c r="D45" s="11">
         <v>52.6</v>
       </c>
       <c r="E45" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="F45" s="26">
+      <c r="F45" s="12">
         <v>0</v>
       </c>
     </row>
@@ -2820,13 +2783,13 @@
       <c r="B46" s="14" t="s">
         <v>118</v>
       </c>
-      <c r="D46" s="25">
+      <c r="D46" s="11">
         <v>33.380000000000003</v>
       </c>
       <c r="E46" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="F46" s="26">
+      <c r="F46" s="12">
         <v>0</v>
       </c>
     </row>
@@ -2835,13 +2798,13 @@
       <c r="B47" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="D47" s="25">
+      <c r="D47" s="11">
         <v>40.730000000000004</v>
       </c>
       <c r="E47" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="F47" s="26">
+      <c r="F47" s="12">
         <v>0</v>
       </c>
     </row>
@@ -2850,13 +2813,13 @@
       <c r="B48" s="14" t="s">
         <v>120</v>
       </c>
-      <c r="D48" s="25">
+      <c r="D48" s="11">
         <v>85.05</v>
       </c>
       <c r="E48" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="F48" s="26">
+      <c r="F48" s="12">
         <v>0</v>
       </c>
     </row>
@@ -2865,13 +2828,13 @@
       <c r="B49" s="14" t="s">
         <v>121</v>
       </c>
-      <c r="D49" s="25">
+      <c r="D49" s="11">
         <v>97.73</v>
       </c>
       <c r="E49" s="19" t="s">
         <v>53</v>
       </c>
-      <c r="F49" s="26">
+      <c r="F49" s="12">
         <v>0</v>
       </c>
     </row>
@@ -2885,13 +2848,13 @@
       <c r="C50" s="2" t="s">
         <v>346</v>
       </c>
-      <c r="D50" s="25">
+      <c r="D50" s="11">
         <v>30.95</v>
       </c>
       <c r="E50" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="F50" s="26">
+      <c r="F50" s="12">
         <v>4.6799999999999837</v>
       </c>
     </row>
@@ -2905,13 +2868,13 @@
       <c r="C51" s="2" t="s">
         <v>347</v>
       </c>
-      <c r="D51" s="25">
+      <c r="D51" s="11">
         <v>25.310000000000002</v>
       </c>
       <c r="E51" s="19" t="s">
         <v>55</v>
       </c>
-      <c r="F51" s="26">
+      <c r="F51" s="12">
         <v>10.921000000000276</v>
       </c>
     </row>
@@ -2925,13 +2888,13 @@
       <c r="C52" s="2" t="s">
         <v>348</v>
       </c>
-      <c r="D52" s="25">
+      <c r="D52" s="11">
         <v>26.55</v>
       </c>
       <c r="E52" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="F52" s="26">
+      <c r="F52" s="12">
         <v>81.549999999997638</v>
       </c>
     </row>
@@ -2945,13 +2908,13 @@
       <c r="C53" s="2" t="s">
         <v>349</v>
       </c>
-      <c r="D53" s="25">
+      <c r="D53" s="11">
         <v>37.869999999999997</v>
       </c>
       <c r="E53" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="F53" s="26">
+      <c r="F53" s="12">
         <v>-1.0000000018073329E-3</v>
       </c>
     </row>
@@ -2965,13 +2928,13 @@
       <c r="C54" s="2" t="s">
         <v>352</v>
       </c>
-      <c r="D54" s="25">
+      <c r="D54" s="11">
         <v>22.59</v>
       </c>
       <c r="E54" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="F54" s="26">
+      <c r="F54" s="12">
         <v>143.72999999999942</v>
       </c>
     </row>
@@ -2985,13 +2948,13 @@
       <c r="C55" s="2" t="s">
         <v>353</v>
       </c>
-      <c r="D55" s="25">
+      <c r="D55" s="11">
         <v>33.380000000000003</v>
       </c>
       <c r="E55" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="F55" s="26">
+      <c r="F55" s="12">
         <v>105.33000000001158</v>
       </c>
     </row>
@@ -3000,13 +2963,13 @@
       <c r="B56" s="14" t="s">
         <v>128</v>
       </c>
-      <c r="D56" s="25">
+      <c r="D56" s="11">
         <v>71.77</v>
       </c>
       <c r="E56" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="F56" s="26">
+      <c r="F56" s="12">
         <v>0</v>
       </c>
     </row>
@@ -3015,13 +2978,13 @@
       <c r="B57" s="14" t="s">
         <v>129</v>
       </c>
-      <c r="D57" s="25">
+      <c r="D57" s="11">
         <v>68.930000000000007</v>
       </c>
       <c r="E57" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="F57" s="26">
+      <c r="F57" s="12">
         <v>0</v>
       </c>
     </row>
@@ -3035,13 +2998,13 @@
       <c r="C58" s="2" t="s">
         <v>354</v>
       </c>
-      <c r="D58" s="25">
+      <c r="D58" s="11">
         <v>47.94</v>
       </c>
       <c r="E58" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="F58" s="26">
+      <c r="F58" s="12">
         <v>62.399999999999942</v>
       </c>
     </row>
@@ -3055,13 +3018,13 @@
       <c r="C59" s="2" t="s">
         <v>354</v>
       </c>
-      <c r="D59" s="25">
+      <c r="D59" s="11">
         <v>25.18</v>
       </c>
       <c r="E59" s="19" t="s">
         <v>63</v>
       </c>
-      <c r="F59" s="26">
+      <c r="F59" s="12">
         <v>0</v>
       </c>
     </row>
@@ -3075,13 +3038,13 @@
       <c r="C60" s="2" t="s">
         <v>355</v>
       </c>
-      <c r="D60" s="25">
+      <c r="D60" s="11">
         <v>39.07</v>
       </c>
       <c r="E60" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="F60" s="26">
+      <c r="F60" s="12">
         <v>0</v>
       </c>
     </row>
@@ -3095,13 +3058,13 @@
       <c r="C61" s="2" t="s">
         <v>356</v>
       </c>
-      <c r="D61" s="25">
+      <c r="D61" s="11">
         <v>42.52</v>
       </c>
       <c r="E61" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="F61" s="26">
+      <c r="F61" s="12">
         <v>-4.9999999997818456E-3</v>
       </c>
     </row>
@@ -3115,13 +3078,13 @@
       <c r="C62" s="2" t="s">
         <v>354</v>
       </c>
-      <c r="D62" s="25">
+      <c r="D62" s="11">
         <v>39.910000000000004</v>
       </c>
       <c r="E62" s="19" t="s">
         <v>66</v>
       </c>
-      <c r="F62" s="26">
+      <c r="F62" s="12">
         <v>0</v>
       </c>
     </row>
@@ -3130,13 +3093,13 @@
       <c r="B63" s="14" t="s">
         <v>135</v>
       </c>
-      <c r="D63" s="25">
+      <c r="D63" s="11">
         <v>33.730000000000004</v>
       </c>
       <c r="E63" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="F63" s="26">
+      <c r="F63" s="12">
         <v>0</v>
       </c>
     </row>
@@ -3150,13 +3113,13 @@
       <c r="C64" s="2" t="s">
         <v>350</v>
       </c>
-      <c r="D64" s="25">
+      <c r="D64" s="11">
         <v>38.94</v>
       </c>
       <c r="E64" s="19" t="s">
         <v>68</v>
       </c>
-      <c r="F64" s="26">
+      <c r="F64" s="12">
         <v>12.200000000000017</v>
       </c>
     </row>
@@ -3170,13 +3133,13 @@
       <c r="C65" s="2" t="s">
         <v>351</v>
       </c>
-      <c r="D65" s="25">
+      <c r="D65" s="11">
         <v>46.37</v>
       </c>
       <c r="E65" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="F65" s="26">
+      <c r="F65" s="12">
         <v>0</v>
       </c>
     </row>
@@ -3185,13 +3148,13 @@
       <c r="B66" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="D66" s="25">
+      <c r="D66" s="11">
         <v>59.300000000000004</v>
       </c>
       <c r="E66" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="F66" s="26">
+      <c r="F66" s="12">
         <v>0</v>
       </c>
     </row>
@@ -3200,13 +3163,13 @@
       <c r="B67" s="14" t="s">
         <v>139</v>
       </c>
-      <c r="D67" s="25">
+      <c r="D67" s="11">
         <v>88.92</v>
       </c>
       <c r="E67" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="F67" s="26">
+      <c r="F67" s="12">
         <v>0</v>
       </c>
     </row>
@@ -3215,13 +3178,13 @@
       <c r="B68" s="14" t="s">
         <v>140</v>
       </c>
-      <c r="D68" s="25">
+      <c r="D68" s="11">
         <v>118.54</v>
       </c>
       <c r="E68" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="F68" s="26">
+      <c r="F68" s="12">
         <v>0</v>
       </c>
     </row>
@@ -3230,13 +3193,13 @@
       <c r="B69" s="14" t="s">
         <v>141</v>
       </c>
-      <c r="D69" s="25">
+      <c r="D69" s="11">
         <v>185.26</v>
       </c>
       <c r="E69" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="F69" s="26">
+      <c r="F69" s="12">
         <v>0</v>
       </c>
     </row>
@@ -3245,13 +3208,13 @@
       <c r="B70" s="14" t="s">
         <v>142</v>
       </c>
-      <c r="D70" s="25">
+      <c r="D70" s="11">
         <v>222.33</v>
       </c>
       <c r="E70" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="F70" s="26">
+      <c r="F70" s="12">
         <v>0</v>
       </c>
     </row>
@@ -3263,80 +3226,80 @@
       <c r="C71" s="2" t="s">
         <v>357</v>
       </c>
-      <c r="D71" s="27">
+      <c r="D71" s="11">
         <v>0.69000000000000006</v>
       </c>
       <c r="E71" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="F71" s="33">
+      <c r="F71" s="12">
         <v>576.00000000000136</v>
       </c>
-      <c r="G71" s="31"/>
+      <c r="G71" s="10"/>
     </row>
     <row r="72" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A72" s="5"/>
       <c r="B72" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="D72" s="27">
+      <c r="D72" s="11">
         <v>0.54</v>
       </c>
       <c r="E72" s="19" t="s">
         <v>200</v>
       </c>
-      <c r="F72" s="33">
+      <c r="F72" s="12">
         <v>0</v>
       </c>
-      <c r="G72" s="31"/>
+      <c r="G72" s="10"/>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A73" s="5"/>
       <c r="B73" s="16" t="s">
         <v>145</v>
       </c>
-      <c r="D73" s="27">
+      <c r="D73" s="11">
         <v>0.35000000000000003</v>
       </c>
       <c r="E73" s="19" t="s">
         <v>201</v>
       </c>
-      <c r="F73" s="33">
+      <c r="F73" s="12">
         <v>0</v>
       </c>
-      <c r="G73" s="31"/>
+      <c r="G73" s="10"/>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A74" s="5"/>
       <c r="B74" s="16" t="s">
         <v>146</v>
       </c>
-      <c r="D74" s="27">
+      <c r="D74" s="11">
         <v>0.28000000000000003</v>
       </c>
       <c r="E74" s="19" t="s">
         <v>202</v>
       </c>
-      <c r="F74" s="33">
+      <c r="F74" s="12">
         <v>0</v>
       </c>
-      <c r="G74" s="31"/>
+      <c r="G74" s="10"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A75" s="5"/>
       <c r="B75" s="16" t="s">
         <v>147</v>
       </c>
-      <c r="D75" s="27">
+      <c r="D75" s="11">
         <v>0.64</v>
       </c>
       <c r="E75" s="19" t="s">
         <v>203</v>
       </c>
-      <c r="F75" s="33">
+      <c r="F75" s="12">
         <v>0</v>
       </c>
-      <c r="G75" s="31"/>
+      <c r="G75" s="10"/>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A76" s="5" t="s">
@@ -3348,16 +3311,16 @@
       <c r="C76" s="17" t="s">
         <v>358</v>
       </c>
-      <c r="D76" s="27">
+      <c r="D76" s="11">
         <v>1.33</v>
       </c>
       <c r="E76" s="19" t="s">
         <v>204</v>
       </c>
-      <c r="F76" s="33">
+      <c r="F76" s="12">
         <v>179</v>
       </c>
-      <c r="G76" s="31"/>
+      <c r="G76" s="10"/>
     </row>
     <row r="77" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A77" s="5" t="s">
@@ -3369,16 +3332,16 @@
       <c r="C77" s="2" t="s">
         <v>359</v>
       </c>
-      <c r="D77" s="27">
+      <c r="D77" s="11">
         <v>1.49</v>
       </c>
       <c r="E77" s="19" t="s">
         <v>205</v>
       </c>
-      <c r="F77" s="33">
+      <c r="F77" s="12">
         <v>151</v>
       </c>
-      <c r="G77" s="31"/>
+      <c r="G77" s="10"/>
     </row>
     <row r="78" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A78" s="5" t="s">
@@ -3390,16 +3353,16 @@
       <c r="C78" s="17" t="s">
         <v>362</v>
       </c>
-      <c r="D78" s="27">
+      <c r="D78" s="11">
         <v>1.6300000000000001</v>
       </c>
       <c r="E78" s="19" t="s">
         <v>206</v>
       </c>
-      <c r="F78" s="33">
+      <c r="F78" s="12">
         <v>302</v>
       </c>
-      <c r="G78" s="31"/>
+      <c r="G78" s="10"/>
     </row>
     <row r="79" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A79" s="5" t="s">
@@ -3411,16 +3374,16 @@
       <c r="C79" s="2" t="s">
         <v>364</v>
       </c>
-      <c r="D79" s="27">
+      <c r="D79" s="11">
         <v>1.82</v>
       </c>
       <c r="E79" s="19" t="s">
         <v>207</v>
       </c>
-      <c r="F79" s="33">
+      <c r="F79" s="12">
         <v>101</v>
       </c>
-      <c r="G79" s="31"/>
+      <c r="G79" s="10"/>
     </row>
     <row r="80" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A80" s="5" t="s">
@@ -3432,16 +3395,16 @@
       <c r="C80" s="17" t="s">
         <v>366</v>
       </c>
-      <c r="D80" s="27">
+      <c r="D80" s="11">
         <v>1.96</v>
       </c>
       <c r="E80" s="19" t="s">
         <v>208</v>
       </c>
-      <c r="F80" s="33">
+      <c r="F80" s="12">
         <v>59</v>
       </c>
-      <c r="G80" s="31"/>
+      <c r="G80" s="10"/>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A81" s="5" t="s">
@@ -3453,16 +3416,16 @@
       <c r="C81" s="2" t="s">
         <v>372</v>
       </c>
-      <c r="D81" s="27">
+      <c r="D81" s="11">
         <v>2.13</v>
       </c>
       <c r="E81" s="19" t="s">
         <v>209</v>
       </c>
-      <c r="F81" s="33">
+      <c r="F81" s="12">
         <v>156</v>
       </c>
-      <c r="G81" s="31"/>
+      <c r="G81" s="10"/>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A82" s="5" t="s">
@@ -3474,16 +3437,16 @@
       <c r="C82" s="17" t="s">
         <v>374</v>
       </c>
-      <c r="D82" s="27">
+      <c r="D82" s="11">
         <v>2.29</v>
       </c>
       <c r="E82" s="19" t="s">
         <v>210</v>
       </c>
-      <c r="F82" s="33">
+      <c r="F82" s="12">
         <v>138</v>
       </c>
-      <c r="G82" s="31"/>
+      <c r="G82" s="10"/>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A83" s="5" t="s">
@@ -3495,16 +3458,16 @@
       <c r="C83" s="2" t="s">
         <v>373</v>
       </c>
-      <c r="D83" s="27">
+      <c r="D83" s="11">
         <v>2.4700000000000002</v>
       </c>
       <c r="E83" s="19" t="s">
         <v>211</v>
       </c>
-      <c r="F83" s="33">
+      <c r="F83" s="12">
         <v>2</v>
       </c>
-      <c r="G83" s="31"/>
+      <c r="G83" s="10"/>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A84" s="5" t="s">
@@ -3516,18 +3479,18 @@
       <c r="C84" s="17" t="s">
         <v>375</v>
       </c>
-      <c r="D84" s="27">
+      <c r="D84" s="11">
         <v>2.61</v>
       </c>
       <c r="E84" s="19" t="s">
         <v>212</v>
       </c>
-      <c r="F84" s="33">
+      <c r="F84" s="12">
         <v>0</v>
       </c>
-      <c r="G84" s="31"/>
-    </row>
-    <row r="85" spans="1:7" s="29" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="G84" s="10"/>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A85" s="5" t="s">
         <v>303</v>
       </c>
@@ -3537,16 +3500,16 @@
       <c r="C85" s="17" t="s">
         <v>462</v>
       </c>
-      <c r="D85" s="32">
+      <c r="D85" s="11">
         <v>1.33</v>
       </c>
-      <c r="E85" s="30" t="s">
+      <c r="E85" s="10" t="s">
         <v>461</v>
       </c>
-      <c r="F85" s="33">
+      <c r="F85" s="12">
         <v>167</v>
       </c>
-      <c r="G85" s="31"/>
+      <c r="G85" s="10"/>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A86" s="5" t="s">
@@ -3558,16 +3521,16 @@
       <c r="C86" s="2" t="s">
         <v>367</v>
       </c>
-      <c r="D86" s="27">
+      <c r="D86" s="11">
         <v>1.59</v>
       </c>
       <c r="E86" s="19" t="s">
         <v>213</v>
       </c>
-      <c r="F86" s="33">
+      <c r="F86" s="12">
         <v>-3</v>
       </c>
-      <c r="G86" s="31"/>
+      <c r="G86" s="10"/>
     </row>
     <row r="87" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A87" s="5" t="s">
@@ -3579,16 +3542,16 @@
       <c r="C87" s="2" t="s">
         <v>368</v>
       </c>
-      <c r="D87" s="27">
+      <c r="D87" s="11">
         <v>1.98</v>
       </c>
       <c r="E87" s="19" t="s">
         <v>214</v>
       </c>
-      <c r="F87" s="33">
+      <c r="F87" s="12">
         <v>0</v>
       </c>
-      <c r="G87" s="31"/>
+      <c r="G87" s="10"/>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A88" s="5" t="s">
@@ -3600,32 +3563,32 @@
       <c r="C88" s="2" t="s">
         <v>369</v>
       </c>
-      <c r="D88" s="27">
+      <c r="D88" s="11">
         <v>2.38</v>
       </c>
       <c r="E88" s="19" t="s">
         <v>215</v>
       </c>
-      <c r="F88" s="33">
+      <c r="F88" s="12">
         <v>-10</v>
       </c>
-      <c r="G88" s="31"/>
+      <c r="G88" s="10"/>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A89" s="5"/>
       <c r="B89" s="16" t="s">
         <v>160</v>
       </c>
-      <c r="D89" s="27">
+      <c r="D89" s="11">
         <v>2.7600000000000002</v>
       </c>
       <c r="E89" s="19" t="s">
         <v>216</v>
       </c>
-      <c r="F89" s="33">
+      <c r="F89" s="12">
         <v>0</v>
       </c>
-      <c r="G89" s="31"/>
+      <c r="G89" s="10"/>
     </row>
     <row r="90" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A90" s="5" t="s">
@@ -3637,16 +3600,16 @@
       <c r="C90" s="2" t="s">
         <v>360</v>
       </c>
-      <c r="D90" s="27">
+      <c r="D90" s="11">
         <v>1.31</v>
       </c>
       <c r="E90" s="19" t="s">
         <v>217</v>
       </c>
-      <c r="F90" s="33">
+      <c r="F90" s="12">
         <v>-11</v>
       </c>
-      <c r="G90" s="31"/>
+      <c r="G90" s="10"/>
     </row>
     <row r="91" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A91" s="5" t="s">
@@ -3658,16 +3621,16 @@
       <c r="C91" s="2" t="s">
         <v>361</v>
       </c>
-      <c r="D91" s="27">
+      <c r="D91" s="11">
         <v>3.12</v>
       </c>
       <c r="E91" s="19" t="s">
         <v>218</v>
       </c>
-      <c r="F91" s="33">
+      <c r="F91" s="12">
         <v>50</v>
       </c>
-      <c r="G91" s="31"/>
+      <c r="G91" s="10"/>
     </row>
     <row r="92" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A92" s="5" t="s">
@@ -3679,16 +3642,16 @@
       <c r="C92" s="2" t="s">
         <v>363</v>
       </c>
-      <c r="D92" s="27">
+      <c r="D92" s="11">
         <v>3.5100000000000002</v>
       </c>
       <c r="E92" s="19" t="s">
         <v>219</v>
       </c>
-      <c r="F92" s="33">
+      <c r="F92" s="12">
         <v>7</v>
       </c>
-      <c r="G92" s="31"/>
+      <c r="G92" s="10"/>
     </row>
     <row r="93" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A93" s="5" t="s">
@@ -3700,16 +3663,16 @@
       <c r="C93" s="2" t="s">
         <v>365</v>
       </c>
-      <c r="D93" s="27">
+      <c r="D93" s="11">
         <v>3.91</v>
       </c>
       <c r="E93" s="19" t="s">
         <v>220</v>
       </c>
-      <c r="F93" s="33">
+      <c r="F93" s="12">
         <v>112</v>
       </c>
-      <c r="G93" s="31"/>
+      <c r="G93" s="10"/>
     </row>
     <row r="94" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A94" s="5" t="s">
@@ -3721,16 +3684,16 @@
       <c r="C94" s="2" t="s">
         <v>370</v>
       </c>
-      <c r="D94" s="27">
+      <c r="D94" s="11">
         <v>4.3100000000000005</v>
       </c>
       <c r="E94" s="19" t="s">
         <v>221</v>
       </c>
-      <c r="F94" s="33">
+      <c r="F94" s="12">
         <v>74</v>
       </c>
-      <c r="G94" s="31"/>
+      <c r="G94" s="10"/>
     </row>
     <row r="95" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A95" s="5" t="s">
@@ -3742,16 +3705,16 @@
       <c r="C95" s="2" t="s">
         <v>371</v>
       </c>
-      <c r="D95" s="27">
+      <c r="D95" s="11">
         <v>4.68</v>
       </c>
       <c r="E95" s="19" t="s">
         <v>222</v>
       </c>
-      <c r="F95" s="33">
+      <c r="F95" s="12">
         <v>75</v>
       </c>
-      <c r="G95" s="31"/>
+      <c r="G95" s="10"/>
     </row>
     <row r="96" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A96" s="5" t="s">
@@ -3763,16 +3726,16 @@
       <c r="C96" s="2" t="s">
         <v>381</v>
       </c>
-      <c r="D96" s="27">
+      <c r="D96" s="11">
         <v>5.07</v>
       </c>
       <c r="E96" s="19" t="s">
         <v>223</v>
       </c>
-      <c r="F96" s="33">
+      <c r="F96" s="12">
         <v>124</v>
       </c>
-      <c r="G96" s="31"/>
+      <c r="G96" s="10"/>
     </row>
     <row r="97" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A97" s="5" t="s">
@@ -3784,32 +3747,32 @@
       <c r="C97" s="2" t="s">
         <v>382</v>
       </c>
-      <c r="D97" s="27">
+      <c r="D97" s="11">
         <v>5.47</v>
       </c>
       <c r="E97" s="19" t="s">
         <v>224</v>
       </c>
-      <c r="F97" s="33">
+      <c r="F97" s="12">
         <v>28</v>
       </c>
-      <c r="G97" s="31"/>
+      <c r="G97" s="10"/>
     </row>
     <row r="98" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A98" s="5"/>
       <c r="B98" s="16" t="s">
         <v>169</v>
       </c>
-      <c r="D98" s="27">
+      <c r="D98" s="11">
         <v>5.87</v>
       </c>
       <c r="E98" s="19" t="s">
         <v>225</v>
       </c>
-      <c r="F98" s="33">
+      <c r="F98" s="12">
         <v>91</v>
       </c>
-      <c r="G98" s="31"/>
+      <c r="G98" s="10"/>
     </row>
     <row r="99" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A99" s="5" t="s">
@@ -3821,16 +3784,16 @@
       <c r="C99" s="2" t="s">
         <v>376</v>
       </c>
-      <c r="D99" s="27">
+      <c r="D99" s="11">
         <v>1.69</v>
       </c>
       <c r="E99" s="19" t="s">
         <v>226</v>
       </c>
-      <c r="F99" s="33">
+      <c r="F99" s="12">
         <v>77</v>
       </c>
-      <c r="G99" s="31"/>
+      <c r="G99" s="10"/>
     </row>
     <row r="100" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A100" s="5" t="s">
@@ -3842,16 +3805,16 @@
       <c r="C100" s="2" t="s">
         <v>378</v>
       </c>
-      <c r="D100" s="27">
+      <c r="D100" s="11">
         <v>3.98</v>
       </c>
       <c r="E100" s="19" t="s">
         <v>227</v>
       </c>
-      <c r="F100" s="33">
+      <c r="F100" s="12">
         <v>60</v>
       </c>
-      <c r="G100" s="31"/>
+      <c r="G100" s="10"/>
     </row>
     <row r="101" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A101" s="5" t="s">
@@ -3863,16 +3826,16 @@
       <c r="C101" s="2" t="s">
         <v>379</v>
       </c>
-      <c r="D101" s="27">
+      <c r="D101" s="11">
         <v>5.12</v>
       </c>
       <c r="E101" s="19" t="s">
         <v>228</v>
       </c>
-      <c r="F101" s="33">
+      <c r="F101" s="12">
         <v>52</v>
       </c>
-      <c r="G101" s="31"/>
+      <c r="G101" s="10"/>
     </row>
     <row r="102" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A102" s="5" t="s">
@@ -3884,32 +3847,32 @@
       <c r="C102" s="2" t="s">
         <v>380</v>
       </c>
-      <c r="D102" s="27">
+      <c r="D102" s="11">
         <v>5.94</v>
       </c>
       <c r="E102" s="19" t="s">
         <v>229</v>
       </c>
-      <c r="F102" s="33">
+      <c r="F102" s="12">
         <v>58</v>
       </c>
-      <c r="G102" s="31"/>
+      <c r="G102" s="10"/>
     </row>
     <row r="103" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A103" s="5"/>
       <c r="B103" s="16" t="s">
         <v>174</v>
       </c>
-      <c r="D103" s="27">
+      <c r="D103" s="11">
         <v>6.92</v>
       </c>
       <c r="E103" s="19" t="s">
         <v>230</v>
       </c>
-      <c r="F103" s="33">
+      <c r="F103" s="12">
         <v>0</v>
       </c>
-      <c r="G103" s="31"/>
+      <c r="G103" s="10"/>
     </row>
     <row r="104" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A104" s="5" t="s">
@@ -3921,16 +3884,16 @@
       <c r="C104" s="2" t="s">
         <v>377</v>
       </c>
-      <c r="D104" s="27">
+      <c r="D104" s="11">
         <v>2.13</v>
       </c>
       <c r="E104" s="19" t="s">
         <v>231</v>
       </c>
-      <c r="F104" s="33">
+      <c r="F104" s="12">
         <v>21</v>
       </c>
-      <c r="G104" s="31"/>
+      <c r="G104" s="10"/>
     </row>
     <row r="105" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A105" s="5" t="s">
@@ -3942,16 +3905,16 @@
       <c r="C105" s="2" t="s">
         <v>383</v>
       </c>
-      <c r="D105" s="27">
+      <c r="D105" s="11">
         <v>5.1100000000000003</v>
       </c>
       <c r="E105" s="19" t="s">
         <v>232</v>
       </c>
-      <c r="F105" s="33">
+      <c r="F105" s="12">
         <v>130</v>
       </c>
-      <c r="G105" s="31"/>
+      <c r="G105" s="10"/>
     </row>
     <row r="106" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A106" s="5" t="s">
@@ -3963,16 +3926,16 @@
       <c r="C106" s="2" t="s">
         <v>393</v>
       </c>
-      <c r="D106" s="27">
+      <c r="D106" s="11">
         <v>5.76</v>
       </c>
       <c r="E106" s="19" t="s">
         <v>233</v>
       </c>
-      <c r="F106" s="33">
+      <c r="F106" s="12">
         <v>66</v>
       </c>
-      <c r="G106" s="31"/>
+      <c r="G106" s="10"/>
     </row>
     <row r="107" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A107" s="5" t="s">
@@ -3984,16 +3947,16 @@
       <c r="C107" s="2" t="s">
         <v>394</v>
       </c>
-      <c r="D107" s="27">
+      <c r="D107" s="11">
         <v>6.3900000000000006</v>
       </c>
       <c r="E107" s="19" t="s">
         <v>234</v>
       </c>
-      <c r="F107" s="33">
+      <c r="F107" s="12">
         <v>47</v>
       </c>
-      <c r="G107" s="31"/>
+      <c r="G107" s="10"/>
     </row>
     <row r="108" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A108" s="5" t="s">
@@ -4005,16 +3968,16 @@
       <c r="C108" s="2" t="s">
         <v>395</v>
       </c>
-      <c r="D108" s="27">
+      <c r="D108" s="11">
         <v>7.03</v>
       </c>
       <c r="E108" s="19" t="s">
         <v>235</v>
       </c>
-      <c r="F108" s="33">
+      <c r="F108" s="12">
         <v>104</v>
       </c>
-      <c r="G108" s="31"/>
+      <c r="G108" s="10"/>
     </row>
     <row r="109" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A109" s="5" t="s">
@@ -4026,16 +3989,16 @@
       <c r="C109" s="2" t="s">
         <v>396</v>
       </c>
-      <c r="D109" s="27">
+      <c r="D109" s="11">
         <v>7.68</v>
       </c>
       <c r="E109" s="19" t="s">
         <v>236</v>
       </c>
-      <c r="F109" s="33">
+      <c r="F109" s="12">
         <v>169</v>
       </c>
-      <c r="G109" s="31"/>
+      <c r="G109" s="10"/>
     </row>
     <row r="110" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A110" s="5" t="s">
@@ -4047,16 +4010,16 @@
       <c r="C110" s="2" t="s">
         <v>397</v>
       </c>
-      <c r="D110" s="27">
+      <c r="D110" s="11">
         <v>8.31</v>
       </c>
       <c r="E110" s="19" t="s">
         <v>237</v>
       </c>
-      <c r="F110" s="33">
+      <c r="F110" s="12">
         <v>23</v>
       </c>
-      <c r="G110" s="31"/>
+      <c r="G110" s="10"/>
     </row>
     <row r="111" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A111" s="5" t="s">
@@ -4068,32 +4031,32 @@
       <c r="C111" s="2" t="s">
         <v>398</v>
       </c>
-      <c r="D111" s="27">
+      <c r="D111" s="11">
         <v>8.9500000000000011</v>
       </c>
       <c r="E111" s="19" t="s">
         <v>238</v>
       </c>
-      <c r="F111" s="33">
+      <c r="F111" s="12">
         <v>8</v>
       </c>
-      <c r="G111" s="31"/>
+      <c r="G111" s="10"/>
     </row>
     <row r="112" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A112" s="5"/>
       <c r="B112" s="16" t="s">
         <v>183</v>
       </c>
-      <c r="D112" s="27">
+      <c r="D112" s="11">
         <v>9.61</v>
       </c>
       <c r="E112" s="19" t="s">
         <v>239</v>
       </c>
-      <c r="F112" s="33">
+      <c r="F112" s="12">
         <v>0</v>
       </c>
-      <c r="G112" s="31"/>
+      <c r="G112" s="10"/>
     </row>
     <row r="113" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A113" s="5" t="s">
@@ -4105,16 +4068,16 @@
       <c r="C113" s="2" t="s">
         <v>384</v>
       </c>
-      <c r="D113" s="27">
+      <c r="D113" s="11">
         <v>4.2700000000000005</v>
       </c>
       <c r="E113" s="19" t="s">
         <v>240</v>
       </c>
-      <c r="F113" s="33">
+      <c r="F113" s="12">
         <v>10</v>
       </c>
-      <c r="G113" s="31"/>
+      <c r="G113" s="10"/>
     </row>
     <row r="114" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A114" s="5" t="s">
@@ -4126,16 +4089,16 @@
       <c r="C114" s="2" t="s">
         <v>385</v>
       </c>
-      <c r="D114" s="27">
+      <c r="D114" s="11">
         <v>10.220000000000001</v>
       </c>
       <c r="E114" s="19" t="s">
         <v>241</v>
       </c>
-      <c r="F114" s="33">
+      <c r="F114" s="12">
         <v>18</v>
       </c>
-      <c r="G114" s="31"/>
+      <c r="G114" s="10"/>
     </row>
     <row r="115" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A115" s="5" t="s">
@@ -4147,16 +4110,16 @@
       <c r="C115" s="2" t="s">
         <v>386</v>
       </c>
-      <c r="D115" s="27">
+      <c r="D115" s="11">
         <v>11.5</v>
       </c>
       <c r="E115" s="19" t="s">
         <v>242</v>
       </c>
-      <c r="F115" s="33">
+      <c r="F115" s="12">
         <v>16</v>
       </c>
-      <c r="G115" s="31"/>
+      <c r="G115" s="10"/>
     </row>
     <row r="116" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A116" s="5" t="s">
@@ -4168,16 +4131,16 @@
       <c r="C116" s="2" t="s">
         <v>387</v>
       </c>
-      <c r="D116" s="27">
+      <c r="D116" s="11">
         <v>12.780000000000001</v>
       </c>
       <c r="E116" s="19" t="s">
         <v>243</v>
       </c>
-      <c r="F116" s="33">
+      <c r="F116" s="12">
         <v>2</v>
       </c>
-      <c r="G116" s="31"/>
+      <c r="G116" s="10"/>
     </row>
     <row r="117" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A117" s="5" t="s">
@@ -4189,16 +4152,16 @@
       <c r="C117" s="2" t="s">
         <v>388</v>
       </c>
-      <c r="D117" s="27">
+      <c r="D117" s="11">
         <v>14.07</v>
       </c>
       <c r="E117" s="19" t="s">
         <v>244</v>
       </c>
-      <c r="F117" s="33">
+      <c r="F117" s="12">
         <v>16</v>
       </c>
-      <c r="G117" s="31"/>
+      <c r="G117" s="10"/>
     </row>
     <row r="118" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A118" s="5" t="s">
@@ -4210,16 +4173,16 @@
       <c r="C118" s="2" t="s">
         <v>389</v>
       </c>
-      <c r="D118" s="27">
+      <c r="D118" s="11">
         <v>15.34</v>
       </c>
       <c r="E118" s="19" t="s">
         <v>245</v>
       </c>
-      <c r="F118" s="33">
+      <c r="F118" s="12">
         <v>32</v>
       </c>
-      <c r="G118" s="31"/>
+      <c r="G118" s="10"/>
     </row>
     <row r="119" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A119" s="5" t="s">
@@ -4231,16 +4194,16 @@
       <c r="C119" s="2" t="s">
         <v>390</v>
       </c>
-      <c r="D119" s="27">
+      <c r="D119" s="11">
         <v>16.61</v>
       </c>
       <c r="E119" s="19" t="s">
         <v>246</v>
       </c>
-      <c r="F119" s="33">
+      <c r="F119" s="12">
         <v>25</v>
       </c>
-      <c r="G119" s="31"/>
+      <c r="G119" s="10"/>
     </row>
     <row r="120" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A120" s="5" t="s">
@@ -4252,32 +4215,32 @@
       <c r="C120" s="2" t="s">
         <v>391</v>
       </c>
-      <c r="D120" s="27">
+      <c r="D120" s="11">
         <v>17.88</v>
       </c>
       <c r="E120" s="19" t="s">
         <v>247</v>
       </c>
-      <c r="F120" s="33">
+      <c r="F120" s="12">
         <v>11</v>
       </c>
-      <c r="G120" s="31"/>
+      <c r="G120" s="10"/>
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A121" s="5"/>
       <c r="B121" s="16" t="s">
         <v>192</v>
       </c>
-      <c r="D121" s="27">
+      <c r="D121" s="11">
         <v>19.12</v>
       </c>
       <c r="E121" s="19" t="s">
         <v>248</v>
       </c>
-      <c r="F121" s="33">
+      <c r="F121" s="12">
         <v>0</v>
       </c>
-      <c r="G121" s="31"/>
+      <c r="G121" s="10"/>
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A122" s="5" t="s">
@@ -4289,16 +4252,16 @@
       <c r="C122" s="2" t="s">
         <v>392</v>
       </c>
-      <c r="D122" s="27">
+      <c r="D122" s="11">
         <v>8.02</v>
       </c>
       <c r="E122" s="19" t="s">
         <v>249</v>
       </c>
-      <c r="F122" s="33">
+      <c r="F122" s="12">
         <v>18</v>
       </c>
-      <c r="G122" s="31"/>
+      <c r="G122" s="10"/>
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A123" s="5" t="s">
@@ -4310,16 +4273,16 @@
       <c r="C123" s="2" t="s">
         <v>399</v>
       </c>
-      <c r="D123" s="27">
+      <c r="D123" s="11">
         <v>18.100000000000001</v>
       </c>
       <c r="E123" s="19" t="s">
         <v>250</v>
       </c>
-      <c r="F123" s="33">
+      <c r="F123" s="12">
         <v>26</v>
       </c>
-      <c r="G123" s="31"/>
+      <c r="G123" s="10"/>
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A124" s="5" t="s">
@@ -4331,16 +4294,16 @@
       <c r="C124" s="2" t="s">
         <v>400</v>
       </c>
-      <c r="D124" s="27">
+      <c r="D124" s="11">
         <v>22.64</v>
       </c>
       <c r="E124" s="19" t="s">
         <v>251</v>
       </c>
-      <c r="F124" s="33">
+      <c r="F124" s="12">
         <v>23</v>
       </c>
-      <c r="G124" s="31"/>
+      <c r="G124" s="10"/>
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A125" s="5" t="s">
@@ -4352,16 +4315,16 @@
       <c r="C125" s="2" t="s">
         <v>401</v>
       </c>
-      <c r="D125" s="27">
+      <c r="D125" s="11">
         <v>27.150000000000002</v>
       </c>
       <c r="E125" s="19" t="s">
         <v>252</v>
       </c>
-      <c r="F125" s="33">
+      <c r="F125" s="12">
         <v>15</v>
       </c>
-      <c r="G125" s="31"/>
+      <c r="G125" s="10"/>
     </row>
     <row r="126" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A126" s="5" t="s">
@@ -4373,16 +4336,16 @@
       <c r="C126" s="2" t="s">
         <v>402</v>
       </c>
-      <c r="D126" s="27">
+      <c r="D126" s="11">
         <v>31.69</v>
       </c>
       <c r="E126" s="19" t="s">
         <v>253</v>
       </c>
-      <c r="F126" s="33">
+      <c r="F126" s="12">
         <v>0</v>
       </c>
-      <c r="G126" s="31"/>
+      <c r="G126" s="10"/>
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A127" s="5" t="s">
@@ -4394,32 +4357,32 @@
       <c r="C127" s="2" t="s">
         <v>403</v>
       </c>
-      <c r="D127" s="27">
+      <c r="D127" s="11">
         <v>33.94</v>
       </c>
       <c r="E127" s="19" t="s">
         <v>254</v>
       </c>
-      <c r="F127" s="33">
+      <c r="F127" s="12">
         <v>0</v>
       </c>
-      <c r="G127" s="31"/>
+      <c r="G127" s="10"/>
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A128" s="5"/>
       <c r="B128" s="15" t="s">
         <v>278</v>
       </c>
-      <c r="D128" s="27">
+      <c r="D128" s="11">
         <v>36.22</v>
       </c>
       <c r="E128" s="19" t="s">
         <v>255</v>
       </c>
-      <c r="F128" s="28">
+      <c r="F128" s="12">
         <v>0</v>
       </c>
-      <c r="G128" s="30"/>
+      <c r="G128" s="10"/>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A129" s="5" t="s">
@@ -4431,13 +4394,13 @@
       <c r="C129" s="2" t="s">
         <v>404</v>
       </c>
-      <c r="D129" s="34">
+      <c r="D129" s="11">
         <v>5.12</v>
       </c>
       <c r="E129" s="19" t="s">
         <v>256</v>
       </c>
-      <c r="F129" s="35">
+      <c r="F129" s="12">
         <v>0</v>
       </c>
     </row>
@@ -4451,13 +4414,13 @@
       <c r="C130" s="2" t="s">
         <v>405</v>
       </c>
-      <c r="D130" s="34">
+      <c r="D130" s="11">
         <v>4.07</v>
       </c>
       <c r="E130" s="19" t="s">
         <v>257</v>
       </c>
-      <c r="F130" s="35">
+      <c r="F130" s="12">
         <v>302</v>
       </c>
     </row>
@@ -4471,13 +4434,13 @@
       <c r="C131" s="2" t="s">
         <v>406</v>
       </c>
-      <c r="D131" s="34">
+      <c r="D131" s="11">
         <v>4.53</v>
       </c>
       <c r="E131" s="19" t="s">
         <v>258</v>
       </c>
-      <c r="F131" s="35">
+      <c r="F131" s="12">
         <v>9</v>
       </c>
     </row>
@@ -4491,13 +4454,13 @@
       <c r="C132" s="2" t="s">
         <v>407</v>
       </c>
-      <c r="D132" s="34">
+      <c r="D132" s="11">
         <v>6.7</v>
       </c>
       <c r="E132" s="19" t="s">
         <v>259</v>
       </c>
-      <c r="F132" s="35">
+      <c r="F132" s="12">
         <v>221</v>
       </c>
     </row>
@@ -4511,13 +4474,13 @@
       <c r="C133" s="2" t="s">
         <v>408</v>
       </c>
-      <c r="D133" s="34">
+      <c r="D133" s="11">
         <v>8.31</v>
       </c>
       <c r="E133" s="19" t="s">
         <v>260</v>
       </c>
-      <c r="F133" s="35">
+      <c r="F133" s="12">
         <v>0</v>
       </c>
     </row>
@@ -4531,13 +4494,13 @@
       <c r="C134" s="2" t="s">
         <v>409</v>
       </c>
-      <c r="D134" s="34">
+      <c r="D134" s="11">
         <v>7.8900000000000006</v>
       </c>
       <c r="E134" s="19" t="s">
         <v>261</v>
       </c>
-      <c r="F134" s="35">
+      <c r="F134" s="12">
         <v>373</v>
       </c>
     </row>
@@ -4551,13 +4514,13 @@
       <c r="C135" s="2" t="s">
         <v>410</v>
       </c>
-      <c r="D135" s="34">
+      <c r="D135" s="11">
         <v>9.61</v>
       </c>
       <c r="E135" s="19" t="s">
         <v>262</v>
       </c>
-      <c r="F135" s="35">
+      <c r="F135" s="12">
         <v>0</v>
       </c>
     </row>
@@ -4566,13 +4529,13 @@
       <c r="B136" s="15" t="s">
         <v>286</v>
       </c>
-      <c r="D136" s="34">
+      <c r="D136" s="11">
         <v>3.5500000000000003</v>
       </c>
       <c r="E136" s="19" t="s">
         <v>263</v>
       </c>
-      <c r="F136" s="35">
+      <c r="F136" s="12">
         <v>0</v>
       </c>
     </row>
@@ -4586,13 +4549,13 @@
       <c r="C137" s="2" t="s">
         <v>411</v>
       </c>
-      <c r="D137" s="34">
+      <c r="D137" s="11">
         <v>6.22</v>
       </c>
       <c r="E137" s="19" t="s">
         <v>264</v>
       </c>
-      <c r="F137" s="35">
+      <c r="F137" s="12">
         <v>351</v>
       </c>
     </row>
@@ -4606,13 +4569,13 @@
       <c r="C138" s="2" t="s">
         <v>418</v>
       </c>
-      <c r="D138" s="34">
+      <c r="D138" s="11">
         <v>6.91</v>
       </c>
       <c r="E138" s="19" t="s">
         <v>265</v>
       </c>
-      <c r="F138" s="35">
+      <c r="F138" s="12">
         <v>162</v>
       </c>
     </row>
@@ -4626,13 +4589,13 @@
       <c r="C139" s="2" t="s">
         <v>419</v>
       </c>
-      <c r="D139" s="34">
+      <c r="D139" s="11">
         <v>10.91</v>
       </c>
       <c r="E139" s="19" t="s">
         <v>266</v>
       </c>
-      <c r="F139" s="35">
+      <c r="F139" s="12">
         <v>0</v>
       </c>
     </row>
@@ -4646,13 +4609,13 @@
       <c r="C140" s="2" t="s">
         <v>420</v>
       </c>
-      <c r="D140" s="34">
+      <c r="D140" s="11">
         <v>10.370000000000001</v>
       </c>
       <c r="E140" s="19" t="s">
         <v>267</v>
       </c>
-      <c r="F140" s="35">
+      <c r="F140" s="12">
         <v>223</v>
       </c>
     </row>
@@ -4666,13 +4629,13 @@
       <c r="C141" s="2" t="s">
         <v>421</v>
       </c>
-      <c r="D141" s="34">
+      <c r="D141" s="11">
         <v>13.88</v>
       </c>
       <c r="E141" s="19" t="s">
         <v>268</v>
       </c>
-      <c r="F141" s="35">
+      <c r="F141" s="12">
         <v>143</v>
       </c>
     </row>
@@ -4686,13 +4649,13 @@
       <c r="C142" s="2" t="s">
         <v>422</v>
       </c>
-      <c r="D142" s="34">
+      <c r="D142" s="11">
         <v>9.23</v>
       </c>
       <c r="E142" s="19" t="s">
         <v>269</v>
       </c>
-      <c r="F142" s="35">
+      <c r="F142" s="12">
         <v>0</v>
       </c>
     </row>
@@ -4706,13 +4669,13 @@
       <c r="C143" s="2" t="s">
         <v>423</v>
       </c>
-      <c r="D143" s="34">
+      <c r="D143" s="11">
         <v>11.14</v>
       </c>
       <c r="E143" s="19" t="s">
         <v>270</v>
       </c>
-      <c r="F143" s="35">
+      <c r="F143" s="12">
         <v>0</v>
       </c>
     </row>
@@ -4721,13 +4684,13 @@
       <c r="B144" s="15" t="s">
         <v>294</v>
       </c>
-      <c r="D144" s="34">
+      <c r="D144" s="11">
         <v>3.17</v>
       </c>
       <c r="E144" s="19" t="s">
         <v>271</v>
       </c>
-      <c r="F144" s="35">
+      <c r="F144" s="12">
         <v>0</v>
       </c>
     </row>
@@ -4741,13 +4704,13 @@
       <c r="C145" s="2" t="s">
         <v>412</v>
       </c>
-      <c r="D145" s="34">
+      <c r="D145" s="11">
         <v>7.2</v>
       </c>
       <c r="E145" s="19" t="s">
         <v>272</v>
       </c>
-      <c r="F145" s="35">
+      <c r="F145" s="12">
         <v>0</v>
       </c>
     </row>
@@ -4761,13 +4724,13 @@
       <c r="C146" s="2" t="s">
         <v>413</v>
       </c>
-      <c r="D146" s="34">
+      <c r="D146" s="11">
         <v>18.11</v>
       </c>
       <c r="E146" s="19" t="s">
         <v>273</v>
       </c>
-      <c r="F146" s="35">
+      <c r="F146" s="12">
         <v>0</v>
       </c>
     </row>
@@ -4781,13 +4744,13 @@
       <c r="C147" s="2" t="s">
         <v>414</v>
       </c>
-      <c r="D147" s="34">
+      <c r="D147" s="11">
         <v>11.94</v>
       </c>
       <c r="E147" s="19" t="s">
         <v>274</v>
       </c>
-      <c r="F147" s="35">
+      <c r="F147" s="12">
         <v>99</v>
       </c>
     </row>
@@ -4801,13 +4764,13 @@
       <c r="C148" s="2" t="s">
         <v>415</v>
       </c>
-      <c r="D148" s="34">
+      <c r="D148" s="11">
         <v>15.16</v>
       </c>
       <c r="E148" s="19" t="s">
         <v>275</v>
       </c>
-      <c r="F148" s="35">
+      <c r="F148" s="12">
         <v>47</v>
       </c>
     </row>
@@ -4821,13 +4784,13 @@
       <c r="C149" s="2" t="s">
         <v>416</v>
       </c>
-      <c r="D149" s="34">
+      <c r="D149" s="11">
         <v>13.52</v>
       </c>
       <c r="E149" s="19" t="s">
         <v>276</v>
       </c>
-      <c r="F149" s="35">
+      <c r="F149" s="12">
         <v>106</v>
       </c>
     </row>
@@ -4841,13 +4804,13 @@
       <c r="C150" s="2" t="s">
         <v>417</v>
       </c>
-      <c r="D150" s="34">
+      <c r="D150" s="11">
         <v>24.89</v>
       </c>
       <c r="E150" s="19" t="s">
         <v>277</v>
       </c>
-      <c r="F150" s="35">
+      <c r="F150" s="12">
         <v>0</v>
       </c>
     </row>
@@ -4928,7 +4891,7 @@
         <v>429</v>
       </c>
       <c r="F154" s="12">
-        <v>16</v>
+        <v>12</v>
       </c>
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.3">
@@ -4941,13 +4904,13 @@
       <c r="C155" s="5" t="s">
         <v>460</v>
       </c>
-      <c r="D155" s="36">
+      <c r="D155" s="11">
         <v>9.82</v>
       </c>
       <c r="E155" s="10" t="s">
         <v>438</v>
       </c>
-      <c r="F155" s="37">
+      <c r="F155" s="12">
         <v>1</v>
       </c>
     </row>
@@ -4961,13 +4924,13 @@
       <c r="C156" s="5" t="s">
         <v>460</v>
       </c>
-      <c r="D156" s="36">
+      <c r="D156" s="11">
         <v>9.82</v>
       </c>
       <c r="E156" s="10" t="s">
         <v>439</v>
       </c>
-      <c r="F156" s="37">
+      <c r="F156" s="12">
         <v>0</v>
       </c>
     </row>
@@ -4981,13 +4944,13 @@
       <c r="C157" s="5" t="s">
         <v>460</v>
       </c>
-      <c r="D157" s="36">
+      <c r="D157" s="11">
         <v>9.82</v>
       </c>
       <c r="E157" s="10" t="s">
         <v>440</v>
       </c>
-      <c r="F157" s="37">
+      <c r="F157" s="12">
         <v>0</v>
       </c>
     </row>
@@ -5001,13 +4964,13 @@
       <c r="C158" s="5" t="s">
         <v>460</v>
       </c>
-      <c r="D158" s="36">
+      <c r="D158" s="11">
         <v>9.82</v>
       </c>
       <c r="E158" s="10" t="s">
         <v>441</v>
       </c>
-      <c r="F158" s="37">
+      <c r="F158" s="12">
         <v>2</v>
       </c>
     </row>
@@ -5021,13 +4984,13 @@
       <c r="C159" s="5" t="s">
         <v>460</v>
       </c>
-      <c r="D159" s="36">
+      <c r="D159" s="11">
         <v>9.82</v>
       </c>
       <c r="E159" s="10" t="s">
         <v>442</v>
       </c>
-      <c r="F159" s="37">
+      <c r="F159" s="12">
         <v>0</v>
       </c>
     </row>
@@ -5041,13 +5004,13 @@
       <c r="C160" s="5" t="s">
         <v>460</v>
       </c>
-      <c r="D160" s="36">
+      <c r="D160" s="11">
         <v>9.82</v>
       </c>
       <c r="E160" s="10" t="s">
         <v>443</v>
       </c>
-      <c r="F160" s="37">
+      <c r="F160" s="12">
         <v>0</v>
       </c>
     </row>
@@ -5061,13 +5024,13 @@
       <c r="C161" s="5" t="s">
         <v>458</v>
       </c>
-      <c r="D161" s="36">
+      <c r="D161" s="11">
         <v>6.3</v>
       </c>
       <c r="E161" s="10" t="s">
         <v>444</v>
       </c>
-      <c r="F161" s="37">
+      <c r="F161" s="12">
         <v>4</v>
       </c>
     </row>

</xml_diff>